<commit_message>
Added an optical permittivity the materials database
</commit_message>
<xml_diff>
--- a/PDielec/MaterialsDataBase.xlsx
+++ b/PDielec/MaterialsDataBase.xlsx
@@ -4,7 +4,7 @@
   <fileVersion lastEdited="4" lowestEdited="4" rupBuild="3820"/>
   <workbookPr date1904="0"/>
   <bookViews>
-    <workbookView activeTab="16" windowWidth="12800" windowHeight="8050"/>
+    <workbookView activeTab="15" windowWidth="12800" windowHeight="8050"/>
   </bookViews>
   <sheets>
     <sheet name="Information" sheetId="1" r:id="rId1"/>
@@ -67,7 +67,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="33" count="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="30" count="30">
   <si>
     <t>Information</t>
   </si>
@@ -79,6 +79,9 @@
   </si>
   <si>
     <t>Density:</t>
+  </si>
+  <si>
+    <t>Optical_permittivity:</t>
   </si>
   <si>
     <t>Temperature:</t>
@@ -153,19 +156,7 @@
     <t>Extrapolated values</t>
   </si>
   <si>
-    <t>B</t>
-  </si>
-  <si>
-    <t>C (microns^2)</t>
-  </si>
-  <si>
-    <t>Sellmeier</t>
-  </si>
-  <si>
-    <t>I. H. Malitson, Applied Optics 2, 1103-1107 (1963)</t>
-  </si>
-  <si>
-    <t>Sellmeier coefficients for CaF2, valid 0.15-12 microns</t>
+    <t>Temperature</t>
   </si>
 </sst>
 </file>
@@ -312,7 +303,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:XFD46"/>
+  <dimension ref="A1:XFD47"/>
   <sheetFormatPr defaultColWidth="12.85546875" defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" style="1" width="28.7109375" customWidth="1"/>
@@ -640,15 +631,13 @@
       <c r="N16" s="2"/>
       <c r="O16" s="2"/>
     </row>
-    <row r="17" spans="1:16384" ht="15">
+    <row r="17" spans="1:16384" ht="14.025">
       <c r="A17" s="2"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D17" s="2">
-        <v>25</v>
-      </c>
+      <c r="D17" s="2"/>
       <c r="E17" s="2"/>
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
@@ -667,7 +656,9 @@
       <c r="C18" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D18" s="2"/>
+      <c r="D18" s="2">
+        <v>25</v>
+      </c>
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
@@ -705,10 +696,7 @@
       <c r="C20" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D20" s="2">
-        <f>COUNT(#REF!)</f>
-        <v>0</v>
-      </c>
+      <c r="D20" s="2"/>
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
@@ -727,8 +715,9 @@
       <c r="C21" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D21" s="2" t="s">
-        <v>9</v>
+      <c r="D21" s="2">
+        <f>COUNT(#REF!)</f>
+        <v>0</v>
       </c>
       <c r="E21" s="2"/>
       <c r="F21" s="2"/>
@@ -745,15 +734,11 @@
     <row r="22" spans="1:16384" ht="15">
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>a_vector:</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>A row vector of 3 floating point numbers specifying the a direction of the unit cell in (xyz)</t>
-        </is>
+      <c r="C22" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>10</v>
       </c>
       <c r="E22" s="2"/>
       <c r="F22" s="2"/>
@@ -772,12 +757,12 @@
       <c r="B23" s="2"/>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>b_vector:</t>
+          <t>a_vector:</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>A row vector of 3 floating point numbers specifying the b direction of the unit cell in (xyz)</t>
+          <t>A row vector of 3 floating point numbers specifying the a direction of the unit cell in (xyz)</t>
         </is>
       </c>
       <c r="E23" s="2"/>
@@ -797,12 +782,12 @@
       <c r="B24" s="2"/>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>c_vector:</t>
+          <t>b_vector:</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>A row vector of 3 floating point numbers specifying the c direction of the unit cell in (xyz)</t>
+          <t>A row vector of 3 floating point numbers specifying the b direction of the unit cell in (xyz)</t>
         </is>
       </c>
       <c r="E24" s="2"/>
@@ -820,12 +805,14 @@
     <row r="25" spans="1:16384" ht="15">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
-      <c r="C25" s="2" t="s">
-        <v>10</v>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>c_vector:</t>
+        </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>The length of the a direction of the cell</t>
+          <t>A row vector of 3 floating point numbers specifying the c direction of the unit cell in (xyz)</t>
         </is>
       </c>
       <c r="E25" s="2"/>
@@ -848,7 +835,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>The length of the b direction of the cell</t>
+          <t>The length of the a direction of the cell</t>
         </is>
       </c>
       <c r="E26" s="2"/>
@@ -871,7 +858,7 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>The length of the c direction of the cell</t>
+          <t>The length of the b direction of the cell</t>
         </is>
       </c>
       <c r="E27" s="2"/>
@@ -894,7 +881,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Cell angle alpha</t>
+          <t>The length of the c direction of the cell</t>
         </is>
       </c>
       <c r="E28" s="2"/>
@@ -917,7 +904,7 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Cell angle beta</t>
+          <t>Cell angle alpha</t>
         </is>
       </c>
       <c r="E29" s="2"/>
@@ -940,7 +927,7 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Cell angle gamma</t>
+          <t>Cell angle beta</t>
         </is>
       </c>
       <c r="E30" s="2"/>
@@ -958,8 +945,14 @@
     <row r="31" spans="1:16384" ht="15">
       <c r="A31" s="2"/>
       <c r="B31" s="2"/>
-      <c r="C31" s="2"/>
-      <c r="D31" s="2"/>
+      <c r="C31" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Cell angle gamma</t>
+        </is>
+      </c>
       <c r="E31" s="2"/>
       <c r="F31" s="2"/>
       <c r="G31" s="2"/>
@@ -973,11 +966,7 @@
       <c r="O31" s="2"/>
     </row>
     <row r="32" spans="1:16384" ht="15">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>The Entry: row is required and can contain;</t>
-        </is>
-      </c>
+      <c r="A32" s="2"/>
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
       <c r="D32" s="2"/>
@@ -994,10 +983,12 @@
       <c r="O32" s="2"/>
     </row>
     <row r="33" spans="1:16384" ht="15">
-      <c r="A33" s="2"/>
-      <c r="B33" s="2" t="s">
-        <v>2</v>
-      </c>
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>The Entry: row is required and can contain;</t>
+        </is>
+      </c>
+      <c r="B33" s="2"/>
       <c r="C33" s="2"/>
       <c r="D33" s="2"/>
       <c r="E33" s="2"/>
@@ -1014,10 +1005,8 @@
     </row>
     <row r="34" spans="1:16384" ht="15">
       <c r="A34" s="2"/>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>Tabulated permittivity</t>
-        </is>
+      <c r="B34" s="2" t="s">
+        <v>2</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" s="2"/>
@@ -1035,8 +1024,10 @@
     </row>
     <row r="35" spans="1:16384" ht="15">
       <c r="A35" s="2"/>
-      <c r="B35" s="2" t="s">
-        <v>16</v>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Tabulated permittivity</t>
+        </is>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
@@ -1073,10 +1064,8 @@
     </row>
     <row r="37" spans="1:16384" ht="15">
       <c r="A37" s="2"/>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>Drude-Lorentz</t>
-        </is>
+      <c r="B37" s="2" t="s">
+        <v>18</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" s="2"/>
@@ -1094,8 +1083,10 @@
     </row>
     <row r="38" spans="1:16384" ht="15">
       <c r="A38" s="2"/>
-      <c r="B38" s="2" t="s">
-        <v>18</v>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Drude-Lorentz</t>
+        </is>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" s="2"/>
@@ -1113,7 +1104,9 @@
     </row>
     <row r="39" spans="1:16384" ht="15">
       <c r="A39" s="2"/>
-      <c r="B39" s="2"/>
+      <c r="B39" s="2" t="s">
+        <v>19</v>
+      </c>
       <c r="C39" s="2"/>
       <c r="D39" s="2"/>
       <c r="E39" s="2"/>
@@ -1126,6 +1119,7 @@
       <c r="L39" s="2"/>
       <c r="M39" s="2"/>
       <c r="N39" s="2"/>
+      <c r="O39" s="2"/>
     </row>
     <row r="40" spans="1:16384" ht="15">
       <c r="A40" s="2"/>
@@ -1176,11 +1170,7 @@
       <c r="N42" s="2"/>
     </row>
     <row r="43" spans="1:16384" ht="15">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>Density: row is required and contains the density in g/ml</t>
-        </is>
-      </c>
+      <c r="A43" s="2"/>
       <c r="B43" s="2"/>
       <c r="C43" s="2"/>
       <c r="D43" s="2"/>
@@ -1196,13 +1186,24 @@
       <c r="N43" s="2"/>
     </row>
     <row r="44" spans="1:16384" ht="15">
-      <c r="A44" s="2"/>
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Density: row is required and contains the density in g/ml</t>
+        </is>
+      </c>
       <c r="B44" s="2"/>
       <c r="C44" s="2"/>
       <c r="D44" s="2"/>
       <c r="E44" s="2"/>
       <c r="F44" s="2"/>
       <c r="G44" s="2"/>
+      <c r="H44" s="2"/>
+      <c r="I44" s="2"/>
+      <c r="J44" s="2"/>
+      <c r="K44" s="2"/>
+      <c r="L44" s="2"/>
+      <c r="M44" s="2"/>
+      <c r="N44" s="2"/>
     </row>
     <row r="45" spans="1:16384" ht="15">
       <c r="A45" s="2"/>
@@ -1221,6 +1222,15 @@
       <c r="E46" s="2"/>
       <c r="F46" s="2"/>
       <c r="G46" s="2"/>
+    </row>
+    <row r="47" spans="1:16384" ht="15">
+      <c r="A47" s="2"/>
+      <c r="B47" s="2"/>
+      <c r="C47" s="2"/>
+      <c r="D47" s="2"/>
+      <c r="E47" s="2"/>
+      <c r="F47" s="2"/>
+      <c r="G47" s="2"/>
     </row>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" selectLockedCells="1" sort="0" autoFilter="0" pivotTables="0" selectUnlockedCells="1"/>
@@ -1239,7 +1249,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="C1:XFD7"/>
+  <dimension ref="C1:XFD8"/>
   <sheetFormatPr defaultColWidth="2.42578125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" style="3" width="5.28515625" bestFit="1" customWidth="1"/>
@@ -1254,16 +1264,16 @@
   <sheetData>
     <row r="1" spans="3:16384">
       <c r="C1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G1" t="s">
         <v>1</v>
       </c>
       <c r="H1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="3:16384">
@@ -1281,20 +1291,19 @@
       </c>
     </row>
     <row r="3" spans="3:16384">
-      <c r="G3" t="s">
+      <c r="G3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="H3" t="s">
-        <v>22</v>
+      <c r="H3">
+        <v>2.2200000000000002</v>
       </c>
     </row>
     <row r="4" spans="3:16384">
       <c r="G4" t="s">
         <v>5</v>
       </c>
-      <c r="H4">
-        <f>MIN(A2:A618)</f>
-        <v>0</v>
+      <c r="H4" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="3:16384">
@@ -1302,7 +1311,7 @@
         <v>6</v>
       </c>
       <c r="H5">
-        <f>MAX(A2:A618)</f>
+        <f>MIN(A3:A619)</f>
         <v>0</v>
       </c>
     </row>
@@ -1311,13 +1320,22 @@
         <v>7</v>
       </c>
       <c r="H6">
-        <f>COUNT(A2:A618)</f>
+        <f>MAX(A3:A619)</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="3:16384">
       <c r="G7" t="s">
         <v>8</v>
+      </c>
+      <c r="H7">
+        <f>COUNT(A3:A619)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="3:16384">
+      <c r="G8" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -1337,7 +1355,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="C1:XFD7"/>
+  <dimension ref="C1:XFD8"/>
   <sheetFormatPr defaultColWidth="12.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="16384" style="3" width="12.85546875" bestFit="1" customWidth="1"/>
@@ -1345,16 +1363,16 @@
   <sheetData>
     <row r="1" spans="3:16384">
       <c r="C1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G1" t="s">
         <v>1</v>
       </c>
       <c r="H1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="3:16384">
@@ -1372,20 +1390,19 @@
       </c>
     </row>
     <row r="3" spans="3:16384">
-      <c r="G3" t="s">
+      <c r="G3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="H3" t="s">
-        <v>22</v>
+      <c r="H3">
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="3:16384">
       <c r="G4" t="s">
         <v>5</v>
       </c>
-      <c r="H4">
-        <f>MIN(A2:A618)</f>
-        <v>0</v>
+      <c r="H4" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="3:16384">
@@ -1393,7 +1410,7 @@
         <v>6</v>
       </c>
       <c r="H5">
-        <f>MAX(A2:A618)</f>
+        <f>MIN(A3:A619)</f>
         <v>0</v>
       </c>
     </row>
@@ -1402,7 +1419,7 @@
         <v>7</v>
       </c>
       <c r="H6">
-        <f>COUNT(A2:A618)</f>
+        <f>MAX(A3:A619)</f>
         <v>0</v>
       </c>
     </row>
@@ -1410,7 +1427,16 @@
       <c r="G7" t="s">
         <v>8</v>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="H7">
+        <f>COUNT(A3:A619)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="3:16384">
+      <c r="G8" t="s">
+        <v>9</v>
+      </c>
+      <c r="H8" t="inlineStr">
         <is>
           <t>D . F . Edwards, in Handbook of Optical Constants of Solids, edited by E. D. Palik (Academic, Orlando, 1985), pp. 547-569.</t>
         </is>
@@ -1449,16 +1475,16 @@
   <sheetData>
     <row r="1" spans="1:16384">
       <c r="A1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1" t="s">
         <v>25</v>
-      </c>
-      <c r="B1" t="s">
-        <v>26</v>
-      </c>
-      <c r="C1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D1" t="s">
-        <v>24</v>
       </c>
       <c r="G1" t="s">
         <v>1</v>
@@ -1480,7 +1506,7 @@
         <v>0.56100000000000017</v>
       </c>
       <c r="E2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G2" t="s">
         <v>3</v>
@@ -1502,13 +1528,13 @@
         <v>0.53820000000000012</v>
       </c>
       <c r="E3" t="s">
-        <v>27</v>
-      </c>
-      <c r="G3" t="s">
+        <v>28</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>4</v>
       </c>
       <c r="H3">
-        <v>25</v>
+        <v>1.77</v>
       </c>
     </row>
     <row r="4" spans="1:16384">
@@ -1529,8 +1555,7 @@
         <v>5</v>
       </c>
       <c r="H4">
-        <f>MIN(A2:A170)</f>
-        <v>0</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:16384">
@@ -1551,8 +1576,8 @@
         <v>6</v>
       </c>
       <c r="H5">
-        <f>MAX(A2:A170)</f>
-        <v>40000</v>
+        <f>MIN(A3:A171)</f>
+        <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:16384">
@@ -1573,8 +1598,8 @@
         <v>7</v>
       </c>
       <c r="H6">
-        <f>COUNT(A2:A170)</f>
-        <v>169</v>
+        <f>MAX(A3:A171)</f>
+        <v>44444.444444444445</v>
       </c>
     </row>
     <row r="7" spans="1:16384">
@@ -1594,8 +1619,9 @@
       <c r="G7" t="s">
         <v>8</v>
       </c>
-      <c r="H7" t="s">
-        <v>9</v>
+      <c r="H7">
+        <f>COUNT(A3:A171)</f>
+        <v>169</v>
       </c>
     </row>
     <row r="8" spans="1:16384">
@@ -1611,6 +1637,12 @@
       </c>
       <c r="D8" s="7">
         <v>0.496</v>
+      </c>
+      <c r="G8" t="s">
+        <v>9</v>
+      </c>
+      <c r="H8" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:16384">
@@ -4105,16 +4137,16 @@
   <sheetData>
     <row r="1" spans="1:16384">
       <c r="A1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1" s="9" t="s">
         <v>25</v>
-      </c>
-      <c r="B1" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C1" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="D1" s="9" t="s">
-        <v>24</v>
       </c>
       <c r="G1" t="s">
         <v>1</v>
@@ -4136,7 +4168,7 @@
         <v>2.0655173210161659</v>
       </c>
       <c r="E2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G2" t="s">
         <v>3</v>
@@ -4159,13 +4191,11 @@
       <c r="D3" s="10">
         <v>1.393</v>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Temperature</t>
-        </is>
+      <c r="G3" s="2" t="s">
+        <v>4</v>
       </c>
       <c r="H3">
-        <v>19</v>
+        <v>1.77</v>
       </c>
     </row>
     <row r="4" spans="1:16384">
@@ -4183,11 +4213,10 @@
         <v>1.169</v>
       </c>
       <c r="G4" t="s">
-        <v>5</v>
+        <v>29</v>
       </c>
       <c r="H4">
-        <f>MIN(A2:A170)</f>
-        <v>0</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:16384">
@@ -4208,8 +4237,8 @@
         <v>6</v>
       </c>
       <c r="H5">
-        <f>MAX(A2:A170)</f>
-        <v>450.04500450045009</v>
+        <f>MIN(A3:A171)</f>
+        <v>5.7703404500865547</v>
       </c>
     </row>
     <row r="6" spans="1:16384">
@@ -4230,8 +4259,8 @@
         <v>7</v>
       </c>
       <c r="H6">
-        <f>COUNT(A2:A170)</f>
-        <v>35</v>
+        <f>MAX(A3:A171)</f>
+        <v>450.04500450045009</v>
       </c>
     </row>
     <row r="7" spans="1:16384">
@@ -4248,15 +4277,12 @@
       <c r="D7" s="10">
         <v>0.79200000000000004</v>
       </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Reference</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>M. N. Afsar and J. B. Hasted. Measurements of the optical constants of liquid H2O and D2O between 6 and 450 cm-1 doi.org/10.1364/JOSA.67.000902 J. Opt. Soc. Am.67, 902-904 (1977)</t>
-        </is>
+      <c r="G7" t="s">
+        <v>8</v>
+      </c>
+      <c r="H7">
+        <f>COUNT(A3:A171)</f>
+        <v>34</v>
       </c>
     </row>
     <row r="8" spans="1:16384">
@@ -4272,6 +4298,16 @@
       </c>
       <c r="D8" s="10">
         <v>0.71199999999999997</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>M. N. Afsar and J. B. Hasted. Measurements of the optical constants of liquid H2O and D2O between 6 and 450 cm-1 doi.org/10.1364/JOSA.67.000902 J. Opt. Soc. Am.67, 902-904 (1977)</t>
+        </is>
       </c>
     </row>
     <row r="9" spans="1:16384">
@@ -4727,16 +4763,16 @@
   <sheetData>
     <row r="1" spans="1:16384">
       <c r="A1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1" t="s">
         <v>25</v>
-      </c>
-      <c r="B1" t="s">
-        <v>26</v>
-      </c>
-      <c r="C1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D1" t="s">
-        <v>24</v>
       </c>
       <c r="G1" t="s">
         <v>1</v>
@@ -4758,7 +4794,7 @@
         <v>872</v>
       </c>
       <c r="E2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G2" t="s">
         <v>3</v>
@@ -4780,13 +4816,13 @@
         <v>781.23199999999997</v>
       </c>
       <c r="E3" t="s">
-        <v>27</v>
-      </c>
-      <c r="G3" t="s">
+        <v>28</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="H3" t="s">
-        <v>22</v>
+      <c r="H3">
+        <v>-13</v>
       </c>
     </row>
     <row r="4" spans="1:16384">
@@ -4806,9 +4842,8 @@
       <c r="G4" t="s">
         <v>5</v>
       </c>
-      <c r="H4">
-        <f>MIN(A2:A170)</f>
-        <v>0</v>
+      <c r="H4" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="1:16384">
@@ -4829,8 +4864,8 @@
         <v>6</v>
       </c>
       <c r="H5">
-        <f>MAX(A2:A170)</f>
-        <v>4032258064.516129</v>
+        <f>MIN(A3:A171)</f>
+        <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:16384">
@@ -4851,8 +4886,8 @@
         <v>7</v>
       </c>
       <c r="H6">
-        <f>COUNT(A2:A170)</f>
-        <v>150</v>
+        <f>MAX(A3:A171)</f>
+        <v>4032258064.516129</v>
       </c>
     </row>
     <row r="7" spans="1:16384">
@@ -4872,10 +4907,9 @@
       <c r="G7" t="s">
         <v>8</v>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>1) H.-J. Hagemann, W. Gudat, and C. Kunz. Optical constants from the far infrared to the x-ray region: Mg, Al, Cu, Ag, Au, Bi, C, and Al&lt;sub&gt;2&lt;/sub&gt;O&lt;sub&gt;3&lt;/sub&gt;, &lt;a href=\"https://doi.org/10.1364/JOSA.65.000742\"&gt;&lt;i&gt;J. Opt. Soc. Am.&lt;/i&gt; &lt;b&gt;65&lt;/b&gt;, 742-744 (1975)&lt;/a&gt;&lt;br&gt;2) H.-J. Hagemann, W. Gudat, and C. Kunz. &lt;a href=\"https://refractiveindex.info/download/data/1974/Hagemann 1974 - DESY report SR-74-7.pdf\"&gt;DESY report SR-74/7 (1974)&lt;/a&gt;"</t>
-        </is>
+      <c r="H7">
+        <f>COUNT(A3:A171)</f>
+        <v>149</v>
       </c>
     </row>
     <row r="8" spans="1:16384">
@@ -4891,6 +4925,14 @@
       </c>
       <c r="D8" s="6">
         <v>90.200000000000003</v>
+      </c>
+      <c r="G8" t="s">
+        <v>9</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>1) H.-J. Hagemann, W. Gudat, and C. Kunz. Optical constants from the far infrared to the x-ray region: Mg, Al, Cu, Ag, Au, Bi, C, and Al&lt;sub&gt;2&lt;/sub&gt;O&lt;sub&gt;3&lt;/sub&gt;, &lt;a href=\"https://doi.org/10.1364/JOSA.65.000742\"&gt;&lt;i&gt;J. Opt. Soc. Am.&lt;/i&gt; &lt;b&gt;65&lt;/b&gt;, 742-744 (1975)&lt;/a&gt;&lt;br&gt;2) H.-J. Hagemann, W. Gudat, and C. Kunz. &lt;a href=\"https://refractiveindex.info/download/data/1974/Hagemann 1974 - DESY report SR-74-7.pdf\"&gt;DESY report SR-74/7 (1974)&lt;/a&gt;"</t>
+        </is>
       </c>
     </row>
     <row r="9" spans="1:16384">
@@ -7071,16 +7113,16 @@
   <sheetData>
     <row r="1" spans="1:16384">
       <c r="A1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1" t="s">
         <v>25</v>
-      </c>
-      <c r="B1" t="s">
-        <v>26</v>
-      </c>
-      <c r="C1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D1" t="s">
-        <v>24</v>
       </c>
       <c r="G1" t="s">
         <v>1</v>
@@ -7101,7 +7143,7 @@
         <v>0</v>
       </c>
       <c r="E2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -7125,10 +7167,10 @@
         <v>0.0022935973613894267</v>
       </c>
       <c r="E3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H3">
         <v>25</v>
@@ -7148,12 +7190,11 @@
       <c r="D4" s="11">
         <v>0.027185000000000001</v>
       </c>
-      <c r="G4" t="s">
-        <v>5</v>
+      <c r="G4" s="2" t="s">
+        <v>4</v>
       </c>
       <c r="H4">
-        <f>MIN(A4:A203)</f>
-        <v>200</v>
+        <v>2.1200000000000001</v>
       </c>
     </row>
     <row r="5" spans="1:16384">
@@ -7174,8 +7215,8 @@
         <v>6</v>
       </c>
       <c r="H5">
-        <f>MAX(A4:A203)</f>
-        <v>1428.5714285714287</v>
+        <f>MIN(A5:A204)</f>
+        <v>206.172814052739</v>
       </c>
     </row>
     <row r="6" spans="1:16384">
@@ -7201,8 +7242,8 @@
         <v>7</v>
       </c>
       <c r="H6">
-        <f>COUNT(A4:A172)</f>
-        <v>169</v>
+        <f>MAX(A5:A204)</f>
+        <v>1428.5714285714287</v>
       </c>
     </row>
     <row r="7" spans="1:16384">
@@ -7222,10 +7263,9 @@
       <c r="G7" t="s">
         <v>8</v>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>1) S. Popova, T. Tolstykh, V. Vorobev. Optical characteristics of amorphous quartz in the 1400â€“200 cm&lt;sup&gt;-1&lt;/sup&gt; region, &lt;i&gt;Opt. Spectrosc.&lt;/i&gt; &lt;b&gt;33&lt;/b&gt;, 444â€“445 (1972), as cited in Ref. 2&lt;br&gt;2) R. Kitamura, L. Pilon, M. Jonasz. Optical constants of silica glass from extreme ultraviolet to far infrared at near room temperature, &lt;a href=\"https://doi.org/10.1364/AO.46.008118\"&gt;&lt;i&gt;Appl. Opt.&lt;/i&gt; &lt;b&gt;33&lt;/b&gt;, 8118-8133 (2007)&lt;/a&gt;&lt;br&gt;&lt;sup&gt;*&lt;/sup&gt; Ref. 2 provides a model for calculating optical constants; model parameters are derived by fitting experimental data from Ref. 1.&lt;br&gt;[&lt;a href=\"https://github.com/polyanskiy/refractiveindex.info-scripts/blob/master/scripts/Kitamura%202007%20-%20Fused%20silica.py\"&gt;Calculation script (Python)&lt;/a&gt;]</t>
-        </is>
+      <c r="H7">
+        <f>COUNT(A5:A173)</f>
+        <v>169</v>
       </c>
     </row>
     <row r="8" spans="1:16384">
@@ -7241,6 +7281,14 @@
       </c>
       <c r="D8" s="11">
         <v>0.041008000000000003</v>
+      </c>
+      <c r="G8" t="s">
+        <v>9</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>1) S. Popova, T. Tolstykh, V. Vorobev. Optical characteristics of amorphous quartz in the 1400â€“200 cm&lt;sup&gt;-1&lt;/sup&gt; region, &lt;i&gt;Opt. Spectrosc.&lt;/i&gt; &lt;b&gt;33&lt;/b&gt;, 444â€“445 (1972), as cited in Ref. 2&lt;br&gt;2) R. Kitamura, L. Pilon, M. Jonasz. Optical constants of silica glass from extreme ultraviolet to far infrared at near room temperature, &lt;a href=\"https://doi.org/10.1364/AO.46.008118\"&gt;&lt;i&gt;Appl. Opt.&lt;/i&gt; &lt;b&gt;33&lt;/b&gt;, 8118-8133 (2007)&lt;/a&gt;&lt;br&gt;&lt;sup&gt;*&lt;/sup&gt; Ref. 2 provides a model for calculating optical constants; model parameters are derived by fitting experimental data from Ref. 1.&lt;br&gt;[&lt;a href=\"https://github.com/polyanskiy/refractiveindex.info-scripts/blob/master/scripts/Kitamura%202007%20-%20Fused%20silica.py\"&gt;Calculation script (Python)&lt;/a&gt;]</t>
+        </is>
       </c>
     </row>
     <row r="9" spans="1:16384">
@@ -10201,16 +10249,16 @@
   <sheetData>
     <row r="1" spans="1:16384">
       <c r="A1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1" t="s">
         <v>25</v>
-      </c>
-      <c r="B1" t="s">
-        <v>26</v>
-      </c>
-      <c r="C1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D1" t="s">
-        <v>24</v>
       </c>
       <c r="G1" t="s">
         <v>1</v>
@@ -10231,7 +10279,7 @@
         <v>0.0055999999999999999</v>
       </c>
       <c r="E2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G2" t="s">
         <v>3</v>
@@ -10253,13 +10301,13 @@
         <v>0.0055999999999999999</v>
       </c>
       <c r="E3" t="s">
-        <v>27</v>
-      </c>
-      <c r="G3" t="s">
+        <v>28</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>4</v>
       </c>
       <c r="H3">
-        <v>25</v>
+        <v>2.3799999999999999</v>
       </c>
     </row>
     <row r="4" spans="1:16384">
@@ -10274,14 +10322,13 @@
         <v>0.0055999999999999999</v>
       </c>
       <c r="E4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G4" t="s">
         <v>5</v>
       </c>
       <c r="H4">
-        <f>MIN(A2:A618)</f>
-        <v>0</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:16384">
@@ -10302,8 +10349,8 @@
         <v>6</v>
       </c>
       <c r="H5">
-        <f>MAX(A2:A618)</f>
-        <v>23255.813953488374</v>
+        <f>MIN(A3:A619)</f>
+        <v>100</v>
       </c>
     </row>
     <row r="6" spans="1:16384">
@@ -10324,8 +10371,8 @@
         <v>7</v>
       </c>
       <c r="H6">
-        <f>COUNT(A2:A618)</f>
-        <v>617</v>
+        <f>MAX(A3:A619)</f>
+        <v>23809.523809523809</v>
       </c>
     </row>
     <row r="7" spans="1:16384">
@@ -10345,10 +10392,9 @@
       <c r="G7" t="s">
         <v>8</v>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>1) X. Zhang, J. Qiu, X. Li, J. Zhao, L. Liu. Complex refractive indices measurements of polymers in visible and near-infrared bands, &lt;a href=\"https://doi.org/10.1364/AO.383831\"&gt;&lt;i&gt;Appl. Opt.&lt;/i&gt; &lt;b&gt;59&lt;/b&gt;, 2337-2344 (2020)&lt;/a&gt; (0.4-2 Âµm)&lt;br&gt;2) X. Zhang, J. Qiu, J. Zhao, X. Li, L. Liu. Complex refractive indices measurements of polymers in infrared bands, &lt;a href=\"https://doi.org/10.1016/j.jqsrt.2020.107063\"&gt;&lt;i&gt;J. Quant. Spectrosc. Radiat. Transf.&lt;/i&gt; &lt;b&gt;252&lt;/b&gt;, 107063 (2020)&lt;/a&gt; (2-20 Âµm)"</t>
-        </is>
+      <c r="H7">
+        <f>COUNT(A3:A619)</f>
+        <v>617</v>
       </c>
     </row>
     <row r="8" spans="1:16384">
@@ -10364,6 +10410,14 @@
       </c>
       <c r="D8" s="14">
         <v>0.0098099999999999993</v>
+      </c>
+      <c r="G8" t="s">
+        <v>9</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>1) X. Zhang, J. Qiu, X. Li, J. Zhao, L. Liu. Complex refractive indices measurements of polymers in visible and near-infrared bands, &lt;a href=\"https://doi.org/10.1364/AO.383831\"&gt;&lt;i&gt;Appl. Opt.&lt;/i&gt; &lt;b&gt;59&lt;/b&gt;, 2337-2344 (2020)&lt;/a&gt; (0.4-2 Âµm)&lt;br&gt;2) X. Zhang, J. Qiu, J. Zhao, X. Li, L. Liu. Complex refractive indices measurements of polymers in infrared bands, &lt;a href=\"https://doi.org/10.1016/j.jqsrt.2020.107063\"&gt;&lt;i&gt;J. Quant. Spectrosc. Radiat. Transf.&lt;/i&gt; &lt;b&gt;252&lt;/b&gt;, 107063 (2020)&lt;/a&gt; (2-20 Âµm)"</t>
+        </is>
       </c>
     </row>
     <row r="9" spans="1:16384">
@@ -19578,7 +19632,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr defaultColWidth="40.8" defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="2" style="0" width="6.605317307692307" bestFit="1" customWidth="1"/>
@@ -19588,17 +19642,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B1" t="s">
-        <v>29</v>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>C (microns^2)</t>
+        </is>
       </c>
       <c r="G1" t="s">
         <v>1</v>
       </c>
-      <c r="H1" t="s">
-        <v>30</v>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Sellmeier</t>
+        </is>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -19622,11 +19682,13 @@
       <c r="B3">
         <v>0.01007833</v>
       </c>
-      <c r="G3" t="s">
-        <v>4</v>
-      </c>
-      <c r="H3" t="s">
-        <v>19</v>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Optical permittivity:</t>
+        </is>
+      </c>
+      <c r="H3">
+        <v>2.04</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -19639,8 +19701,8 @@
       <c r="G4" t="s">
         <v>5</v>
       </c>
-      <c r="H4">
-        <v>833</v>
+      <c r="H4" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -19648,7 +19710,7 @@
         <v>6</v>
       </c>
       <c r="H5">
-        <v>66667</v>
+        <v>833</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -19656,20 +19718,32 @@
         <v>7</v>
       </c>
       <c r="H6">
-        <v>0</v>
+        <v>66667</v>
       </c>
     </row>
     <row r="7" spans="1:8">
       <c r="G7" t="s">
         <v>8</v>
       </c>
-      <c r="H7" t="s">
-        <v>31</v>
+      <c r="H7">
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:8">
-      <c r="H8" t="s">
-        <v>32</v>
+      <c r="G8" t="s">
+        <v>9</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>I. H. Malitson, Applied Optics 2, 1103-1107 (1963)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Sellmeier coefficients for CaF2, valid 0.15-12 microns</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -19689,7 +19763,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P15"/>
+  <dimension ref="A1:P16"/>
   <sheetFormatPr defaultColWidth="48" defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" style="0" width="14.28515625" customWidth="1"/>
@@ -19738,7 +19812,7 @@
         <v>1</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I1" s="3"/>
       <c r="J1" s="3"/>
@@ -19801,7 +19875,7 @@
         <v>3.7000000000000002</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H3" s="6">
         <v>4.7605000000000004</v>
@@ -19835,7 +19909,7 @@
         <v>7</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H4" s="6">
         <v>4.7605000000000004</v>
@@ -19869,7 +19943,7 @@
         <v>17.800000000000001</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H5" s="6">
         <v>12.9956</v>
@@ -19905,7 +19979,7 @@
         <v>4</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H6" s="3">
         <v>90</v>
@@ -19935,7 +20009,7 @@
         <v>3.7000000000000002</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H7" s="3">
         <v>90</v>
@@ -19965,7 +20039,7 @@
         <v>7</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H8" s="3">
         <v>120</v>
@@ -19994,11 +20068,11 @@
       <c r="F9" s="4">
         <v>17.800000000000001</v>
       </c>
-      <c r="G9" s="3" t="s">
+      <c r="G9" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="H9" s="3" t="s">
-        <v>19</v>
+      <c r="H9" s="3">
+        <v>3.0800000000000001</v>
       </c>
       <c r="I9" s="3"/>
       <c r="J9" s="3"/>
@@ -20033,8 +20107,8 @@
       <c r="G10" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="H10" s="3">
-        <v>0</v>
+      <c r="H10" s="3" t="s">
+        <v>20</v>
       </c>
       <c r="I10" s="3"/>
       <c r="J10" s="3"/>
@@ -20107,10 +20181,8 @@
       <c r="G13" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="H13" s="3" t="inlineStr">
-        <is>
-          <t>S.C. Lee, S.S. Ng, H. Abu Hassan, Z. Hassan, T. Dumelow</t>
-        </is>
+      <c r="H13" s="3">
+        <v>0</v>
       </c>
       <c r="I13" s="3"/>
       <c r="J13" s="3"/>
@@ -20128,10 +20200,12 @@
       <c r="D14" s="3"/>
       <c r="E14" s="3"/>
       <c r="F14" s="3"/>
-      <c r="G14" s="3"/>
+      <c r="G14" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>Crystal orientation dependence of polarized infrared reflectance response of hexagonal sapphire crystal</t>
+          <t>S.C. Lee, S.S. Ng, H. Abu Hassan, Z. Hassan, T. Dumelow</t>
         </is>
       </c>
       <c r="I14" s="3"/>
@@ -20153,7 +20227,7 @@
       <c r="G15" s="3"/>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>Optical Materials (2014) vol 37, 773-779</t>
+          <t>Crystal orientation dependence of polarized infrared reflectance response of hexagonal sapphire crystal</t>
         </is>
       </c>
       <c r="I15" s="3"/>
@@ -20164,6 +20238,14 @@
       <c r="N15" s="3"/>
       <c r="O15" s="3"/>
       <c r="P15" s="3"/>
+    </row>
+    <row r="16" spans="1:16" ht="14.025">
+      <c r="G16" s="3"/>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>Optical Materials (2014) vol 37, 773-779</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" selectLockedCells="1" sort="0" autoFilter="0" pivotTables="0" selectUnlockedCells="1"/>
@@ -20182,7 +20264,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="C1:XFD7"/>
+  <dimension ref="C1:XFD8"/>
   <sheetFormatPr defaultColWidth="2.42578125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" style="3" width="5.140625" bestFit="1" customWidth="1"/>
@@ -20197,16 +20279,16 @@
   <sheetData>
     <row r="1" spans="3:16384">
       <c r="C1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G1" t="s">
         <v>1</v>
       </c>
       <c r="H1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" spans="3:16384">
@@ -20224,20 +20306,19 @@
       </c>
     </row>
     <row r="3" spans="3:16384">
-      <c r="G3" t="s">
+      <c r="G3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="H3" t="s">
-        <v>22</v>
+      <c r="H3">
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="3:16384">
       <c r="G4" t="s">
         <v>5</v>
       </c>
-      <c r="H4">
-        <f>MIN(A2:A618)</f>
-        <v>0</v>
+      <c r="H4" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="3:16384">
@@ -20245,7 +20326,7 @@
         <v>6</v>
       </c>
       <c r="H5">
-        <f>MAX(A2:A618)</f>
+        <f>MIN(A3:A619)</f>
         <v>0</v>
       </c>
     </row>
@@ -20254,13 +20335,22 @@
         <v>7</v>
       </c>
       <c r="H6">
-        <f>COUNT(A2:A618)</f>
+        <f>MAX(A3:A619)</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="3:16384">
       <c r="G7" t="s">
         <v>8</v>
+      </c>
+      <c r="H7">
+        <f>COUNT(A3:A619)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="3:16384">
+      <c r="G8" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -20280,7 +20370,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="C1:XFD7"/>
+  <dimension ref="C1:XFD8"/>
   <sheetFormatPr defaultColWidth="2.42578125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" style="3" width="5.28515625" bestFit="1" customWidth="1"/>
@@ -20295,16 +20385,16 @@
   <sheetData>
     <row r="1" spans="3:16384">
       <c r="C1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G1" t="s">
         <v>1</v>
       </c>
       <c r="H1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" spans="3:16384">
@@ -20322,20 +20412,19 @@
       </c>
     </row>
     <row r="3" spans="3:16384">
-      <c r="G3" t="s">
+      <c r="G3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="H3" t="s">
-        <v>22</v>
+      <c r="H3">
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="3:16384">
       <c r="G4" t="s">
         <v>5</v>
       </c>
-      <c r="H4">
-        <f>MIN(A2:A618)</f>
-        <v>0</v>
+      <c r="H4" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="3:16384">
@@ -20343,7 +20432,7 @@
         <v>6</v>
       </c>
       <c r="H5">
-        <f>MAX(A2:A618)</f>
+        <f>MIN(A3:A619)</f>
         <v>0</v>
       </c>
     </row>
@@ -20352,13 +20441,22 @@
         <v>7</v>
       </c>
       <c r="H6">
-        <f>COUNT(A2:A618)</f>
+        <f>MAX(A3:A619)</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="3:16384">
       <c r="G7" t="s">
         <v>8</v>
+      </c>
+      <c r="H7">
+        <f>COUNT(A3:A619)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="3:16384">
+      <c r="G8" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -20378,7 +20476,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="C1:XFD7"/>
+  <dimension ref="C1:XFD8"/>
   <sheetFormatPr defaultColWidth="2.42578125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" style="3" width="5.28515625" bestFit="1" customWidth="1"/>
@@ -20393,16 +20491,16 @@
   <sheetData>
     <row r="1" spans="3:16384">
       <c r="C1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G1" t="s">
         <v>1</v>
       </c>
       <c r="H1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" spans="3:16384">
@@ -20420,20 +20518,19 @@
       </c>
     </row>
     <row r="3" spans="3:16384">
-      <c r="G3" t="s">
+      <c r="G3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="H3" t="s">
-        <v>22</v>
+      <c r="H3">
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="3:16384">
       <c r="G4" t="s">
         <v>5</v>
       </c>
-      <c r="H4">
-        <f>MIN(A2:A618)</f>
-        <v>0</v>
+      <c r="H4" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="3:16384">
@@ -20441,7 +20538,7 @@
         <v>6</v>
       </c>
       <c r="H5">
-        <f>MAX(A2:A618)</f>
+        <f>MIN(A3:A619)</f>
         <v>0</v>
       </c>
     </row>
@@ -20450,13 +20547,22 @@
         <v>7</v>
       </c>
       <c r="H6">
-        <f>COUNT(A2:A618)</f>
+        <f>MAX(A3:A619)</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="3:16384">
       <c r="G7" t="s">
         <v>8</v>
+      </c>
+      <c r="H7">
+        <f>COUNT(A3:A619)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="3:16384">
+      <c r="G8" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -20476,7 +20582,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="C1:XFD7"/>
+  <dimension ref="C1:XFD8"/>
   <sheetFormatPr defaultColWidth="2.42578125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" style="3" width="5.28515625" bestFit="1" customWidth="1"/>
@@ -20491,16 +20597,16 @@
   <sheetData>
     <row r="1" spans="3:16384">
       <c r="C1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G1" t="s">
         <v>1</v>
       </c>
       <c r="H1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" spans="3:16384">
@@ -20518,20 +20624,19 @@
       </c>
     </row>
     <row r="3" spans="3:16384">
-      <c r="G3" t="s">
+      <c r="G3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="H3" t="s">
-        <v>22</v>
+      <c r="H3">
+        <v>2.2799999999999998</v>
       </c>
     </row>
     <row r="4" spans="3:16384">
       <c r="G4" t="s">
         <v>5</v>
       </c>
-      <c r="H4">
-        <f>MIN(A2:A618)</f>
-        <v>0</v>
+      <c r="H4" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="3:16384">
@@ -20539,7 +20644,7 @@
         <v>6</v>
       </c>
       <c r="H5">
-        <f>MAX(A2:A618)</f>
+        <f>MIN(A3:A619)</f>
         <v>0</v>
       </c>
     </row>
@@ -20548,13 +20653,22 @@
         <v>7</v>
       </c>
       <c r="H6">
-        <f>COUNT(A2:A618)</f>
+        <f>MAX(A3:A619)</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="3:16384">
       <c r="G7" t="s">
         <v>8</v>
+      </c>
+      <c r="H7">
+        <f>COUNT(A3:A619)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="3:16384">
+      <c r="G8" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -20574,7 +20688,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="C1:XFD7"/>
+  <dimension ref="C1:XFD8"/>
   <sheetFormatPr defaultColWidth="2.42578125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" style="3" width="5.28515625" bestFit="1" customWidth="1"/>
@@ -20589,16 +20703,16 @@
   <sheetData>
     <row r="1" spans="3:16384">
       <c r="C1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G1" t="s">
         <v>1</v>
       </c>
       <c r="H1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" spans="3:16384">
@@ -20616,20 +20730,19 @@
       </c>
     </row>
     <row r="3" spans="3:16384">
-      <c r="G3" t="s">
+      <c r="G3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="H3" t="s">
-        <v>22</v>
+      <c r="H3">
+        <v>2.2999999999999998</v>
       </c>
     </row>
     <row r="4" spans="3:16384">
       <c r="G4" t="s">
         <v>5</v>
       </c>
-      <c r="H4">
-        <f>MIN(A2:A618)</f>
-        <v>0</v>
+      <c r="H4" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="3:16384">
@@ -20637,7 +20750,7 @@
         <v>6</v>
       </c>
       <c r="H5">
-        <f>MAX(A2:A618)</f>
+        <f>MIN(A3:A619)</f>
         <v>0</v>
       </c>
     </row>
@@ -20646,13 +20759,22 @@
         <v>7</v>
       </c>
       <c r="H6">
-        <f>COUNT(A2:A618)</f>
+        <f>MAX(A3:A619)</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="3:16384">
       <c r="G7" t="s">
         <v>8</v>
+      </c>
+      <c r="H7">
+        <f>COUNT(A3:A619)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="3:16384">
+      <c r="G8" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -20672,7 +20794,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="C1:XFD7"/>
+  <dimension ref="C1:XFD8"/>
   <sheetFormatPr defaultColWidth="2.42578125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" style="3" width="5.28515625" bestFit="1" customWidth="1"/>
@@ -20687,16 +20809,16 @@
   <sheetData>
     <row r="1" spans="3:16384">
       <c r="C1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G1" t="s">
         <v>1</v>
       </c>
       <c r="H1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" spans="3:16384">
@@ -20714,20 +20836,19 @@
       </c>
     </row>
     <row r="3" spans="3:16384">
-      <c r="G3" t="s">
+      <c r="G3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="H3" t="s">
-        <v>22</v>
+      <c r="H3">
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="4" spans="3:16384">
       <c r="G4" t="s">
         <v>5</v>
       </c>
-      <c r="H4">
-        <f>MIN(A2:A618)</f>
-        <v>0</v>
+      <c r="H4" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="3:16384">
@@ -20735,7 +20856,7 @@
         <v>6</v>
       </c>
       <c r="H5">
-        <f>MAX(A2:A618)</f>
+        <f>MIN(A3:A619)</f>
         <v>0</v>
       </c>
     </row>
@@ -20744,13 +20865,22 @@
         <v>7</v>
       </c>
       <c r="H6">
-        <f>COUNT(A2:A618)</f>
+        <f>MAX(A3:A619)</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="3:16384">
       <c r="G7" t="s">
         <v>8</v>
+      </c>
+      <c r="H7">
+        <f>COUNT(A3:A619)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="3:16384">
+      <c r="G8" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -20770,7 +20900,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="C1:XFD7"/>
+  <dimension ref="C1:XFD8"/>
   <sheetFormatPr defaultColWidth="2.42578125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" style="3" width="5.28515625" bestFit="1" customWidth="1"/>
@@ -20785,16 +20915,16 @@
   <sheetData>
     <row r="1" spans="3:16384">
       <c r="C1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G1" t="s">
         <v>1</v>
       </c>
       <c r="H1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" spans="3:16384">
@@ -20812,20 +20942,19 @@
       </c>
     </row>
     <row r="3" spans="3:16384">
-      <c r="G3" t="s">
+      <c r="G3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="H3" t="s">
-        <v>22</v>
+      <c r="H3">
+        <v>2.1499999999999999</v>
       </c>
     </row>
     <row r="4" spans="3:16384">
       <c r="G4" t="s">
         <v>5</v>
       </c>
-      <c r="H4">
-        <f>MIN(A2:A618)</f>
-        <v>0</v>
+      <c r="H4" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="3:16384">
@@ -20833,7 +20962,7 @@
         <v>6</v>
       </c>
       <c r="H5">
-        <f>MAX(A2:A618)</f>
+        <f>MIN(A3:A619)</f>
         <v>0</v>
       </c>
     </row>
@@ -20842,13 +20971,22 @@
         <v>7</v>
       </c>
       <c r="H6">
-        <f>COUNT(A2:A618)</f>
+        <f>MAX(A3:A619)</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="3:16384">
       <c r="G7" t="s">
         <v>8</v>
+      </c>
+      <c r="H7">
+        <f>COUNT(A3:A619)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="3:16384">
+      <c r="G8" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added additional values for the Water 19C to allow interpolation
</commit_message>
<xml_diff>
--- a/PDielec/MaterialsDataBase.xlsx
+++ b/PDielec/MaterialsDataBase.xlsx
@@ -4,7 +4,7 @@
   <fileVersion lastEdited="4" lowestEdited="4" rupBuild="3820"/>
   <workbookPr date1904="0"/>
   <bookViews>
-    <workbookView activeTab="15" windowWidth="12800" windowHeight="8050"/>
+    <workbookView activeTab="12" windowWidth="19200" windowHeight="8340"/>
   </bookViews>
   <sheets>
     <sheet name="Information" sheetId="1" r:id="rId1"/>
@@ -67,7 +67,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="30" count="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="29" count="29">
   <si>
     <t>Information</t>
   </si>
@@ -154,9 +154,6 @@
   </si>
   <si>
     <t>Extrapolated values</t>
-  </si>
-  <si>
-    <t>Temperature</t>
   </si>
 </sst>
 </file>
@@ -4122,7 +4119,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:XFD36"/>
+  <dimension ref="A1:XFD54"/>
   <sheetFormatPr defaultColWidth="2.42578125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" style="3" width="13.7109375" bestFit="1" customWidth="1"/>
@@ -4212,8 +4209,10 @@
       <c r="D4" s="10">
         <v>1.169</v>
       </c>
-      <c r="G4" t="s">
-        <v>29</v>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Temperature</t>
+        </is>
       </c>
       <c r="H4">
         <v>19</v>
@@ -4260,7 +4259,7 @@
       </c>
       <c r="H6">
         <f>MAX(A3:A171)</f>
-        <v>450.04500450045009</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="7" spans="1:16384">
@@ -4282,7 +4281,7 @@
       </c>
       <c r="H7">
         <f>COUNT(A3:A171)</f>
-        <v>34</v>
+        <v>52</v>
       </c>
     </row>
     <row r="8" spans="1:16384">
@@ -4727,6 +4726,281 @@
         <v>1.51</v>
       </c>
       <c r="D36" s="10">
+        <v>0.375</v>
+      </c>
+    </row>
+    <row r="37" spans="1:16384">
+      <c r="A37" s="8">
+        <f>10000/B37</f>
+        <v>476.1904761904762</v>
+      </c>
+      <c r="B37">
+        <v>21</v>
+      </c>
+      <c r="C37">
+        <v>1.51</v>
+      </c>
+      <c r="D37">
+        <v>0.375</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Extrapolated</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" spans="1:16384">
+      <c r="A38" s="8">
+        <f>10000/B38</f>
+        <v>500</v>
+      </c>
+      <c r="B38">
+        <v>20</v>
+      </c>
+      <c r="C38">
+        <v>1.51</v>
+      </c>
+      <c r="D38">
+        <v>0.375</v>
+      </c>
+    </row>
+    <row r="39" spans="1:16384">
+      <c r="A39" s="8">
+        <f>10000/B39</f>
+        <v>526.31578947368416</v>
+      </c>
+      <c r="B39">
+        <v>19</v>
+      </c>
+      <c r="C39">
+        <v>1.51</v>
+      </c>
+      <c r="D39">
+        <v>0.375</v>
+      </c>
+    </row>
+    <row r="40" spans="1:16384">
+      <c r="A40" s="8">
+        <f>10000/B40</f>
+        <v>555.55555555555554</v>
+      </c>
+      <c r="B40">
+        <v>18</v>
+      </c>
+      <c r="C40">
+        <v>1.51</v>
+      </c>
+      <c r="D40">
+        <v>0.375</v>
+      </c>
+    </row>
+    <row r="41" spans="1:16384">
+      <c r="A41" s="8">
+        <f>10000/B41</f>
+        <v>588.23529411764707</v>
+      </c>
+      <c r="B41">
+        <v>17</v>
+      </c>
+      <c r="C41">
+        <v>1.51</v>
+      </c>
+      <c r="D41">
+        <v>0.375</v>
+      </c>
+    </row>
+    <row r="42" spans="1:16384">
+      <c r="A42" s="8">
+        <f>10000/B42</f>
+        <v>625</v>
+      </c>
+      <c r="B42">
+        <v>16</v>
+      </c>
+      <c r="C42">
+        <v>1.51</v>
+      </c>
+      <c r="D42">
+        <v>0.375</v>
+      </c>
+    </row>
+    <row r="43" spans="1:16384">
+      <c r="A43" s="8">
+        <f>10000/B43</f>
+        <v>666.66666666666663</v>
+      </c>
+      <c r="B43">
+        <v>15</v>
+      </c>
+      <c r="C43">
+        <v>1.51</v>
+      </c>
+      <c r="D43">
+        <v>0.375</v>
+      </c>
+    </row>
+    <row r="44" spans="1:16384">
+      <c r="A44" s="8">
+        <f>10000/B44</f>
+        <v>714.28571428571433</v>
+      </c>
+      <c r="B44">
+        <v>14</v>
+      </c>
+      <c r="C44">
+        <v>1.51</v>
+      </c>
+      <c r="D44">
+        <v>0.375</v>
+      </c>
+    </row>
+    <row r="45" spans="1:16384">
+      <c r="A45" s="8">
+        <f>10000/B45</f>
+        <v>769.23076923076928</v>
+      </c>
+      <c r="B45">
+        <v>13</v>
+      </c>
+      <c r="C45">
+        <v>1.51</v>
+      </c>
+      <c r="D45">
+        <v>0.375</v>
+      </c>
+    </row>
+    <row r="46" spans="1:16384">
+      <c r="A46" s="8">
+        <f>10000/B46</f>
+        <v>833.33333333333337</v>
+      </c>
+      <c r="B46">
+        <v>12</v>
+      </c>
+      <c r="C46">
+        <v>1.51</v>
+      </c>
+      <c r="D46">
+        <v>0.375</v>
+      </c>
+    </row>
+    <row r="47" spans="1:16384">
+      <c r="A47" s="8">
+        <f>10000/B47</f>
+        <v>909.09090909090912</v>
+      </c>
+      <c r="B47">
+        <v>11</v>
+      </c>
+      <c r="C47">
+        <v>1.51</v>
+      </c>
+      <c r="D47">
+        <v>0.375</v>
+      </c>
+    </row>
+    <row r="48" spans="1:16384">
+      <c r="A48" s="8">
+        <f>10000/B48</f>
+        <v>1000</v>
+      </c>
+      <c r="B48">
+        <v>10</v>
+      </c>
+      <c r="C48">
+        <v>1.51</v>
+      </c>
+      <c r="D48">
+        <v>0.375</v>
+      </c>
+    </row>
+    <row r="49" spans="1:16384">
+      <c r="A49" s="8">
+        <f>10000/B49</f>
+        <v>1111.1111111111111</v>
+      </c>
+      <c r="B49">
+        <v>9</v>
+      </c>
+      <c r="C49">
+        <v>1.51</v>
+      </c>
+      <c r="D49">
+        <v>0.375</v>
+      </c>
+    </row>
+    <row r="50" spans="1:16384">
+      <c r="A50" s="8">
+        <f>10000/B50</f>
+        <v>1250</v>
+      </c>
+      <c r="B50">
+        <v>8</v>
+      </c>
+      <c r="C50">
+        <v>1.51</v>
+      </c>
+      <c r="D50">
+        <v>0.375</v>
+      </c>
+    </row>
+    <row r="51" spans="1:16384">
+      <c r="A51" s="8">
+        <f>10000/B51</f>
+        <v>1428.5714285714287</v>
+      </c>
+      <c r="B51">
+        <v>7</v>
+      </c>
+      <c r="C51">
+        <v>1.51</v>
+      </c>
+      <c r="D51">
+        <v>0.375</v>
+      </c>
+    </row>
+    <row r="52" spans="1:16384">
+      <c r="A52" s="8">
+        <f>10000/B52</f>
+        <v>1666.6666666666667</v>
+      </c>
+      <c r="B52">
+        <v>6</v>
+      </c>
+      <c r="C52">
+        <v>1.51</v>
+      </c>
+      <c r="D52">
+        <v>0.375</v>
+      </c>
+    </row>
+    <row r="53" spans="1:16384">
+      <c r="A53" s="8">
+        <f>10000/B53</f>
+        <v>2000</v>
+      </c>
+      <c r="B53">
+        <v>5</v>
+      </c>
+      <c r="C53">
+        <v>1.51</v>
+      </c>
+      <c r="D53">
+        <v>0.375</v>
+      </c>
+    </row>
+    <row r="54" spans="1:16384">
+      <c r="A54" s="8">
+        <f>10000/B54</f>
+        <v>2500</v>
+      </c>
+      <c r="B54">
+        <v>4</v>
+      </c>
+      <c r="C54">
+        <v>1.51</v>
+      </c>
+      <c r="D54">
         <v>0.375</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Removed optical_permittivity from all entries except the tabulated entries.
</commit_message>
<xml_diff>
--- a/PDielec/MaterialsDataBase.xlsx
+++ b/PDielec/MaterialsDataBase.xlsx
@@ -4,7 +4,7 @@
   <fileVersion lastEdited="4" lowestEdited="4" rupBuild="3820"/>
   <workbookPr date1904="0"/>
   <bookViews>
-    <workbookView activeTab="12" windowWidth="19200" windowHeight="8340"/>
+    <workbookView activeTab="16" windowWidth="19200" windowHeight="8340"/>
   </bookViews>
   <sheets>
     <sheet name="Information" sheetId="1" r:id="rId1"/>
@@ -1288,52 +1288,48 @@
       </c>
     </row>
     <row r="3" spans="3:16384">
-      <c r="G3" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="H3">
-        <v>2.2200000000000002</v>
+      <c r="G3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H3" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="3:16384">
       <c r="G4" t="s">
-        <v>5</v>
-      </c>
-      <c r="H4" t="s">
-        <v>23</v>
+        <v>6</v>
+      </c>
+      <c r="H4">
+        <f>MIN(A3:A619)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="3:16384">
       <c r="G5" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H5">
-        <f>MIN(A3:A619)</f>
+        <f>MAX(A3:A619)</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="3:16384">
       <c r="G6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H6">
-        <f>MAX(A3:A619)</f>
+        <f>COUNT(A3:A619)</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="3:16384">
       <c r="G7" t="s">
-        <v>8</v>
-      </c>
-      <c r="H7">
-        <f>COUNT(A3:A619)</f>
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="3:16384">
-      <c r="G8" t="s">
-        <v>9</v>
-      </c>
+      <c r="G8" s="0"/>
+      <c r="H8" s="0"/>
     </row>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" selectLockedCells="1" sort="0" autoFilter="0" pivotTables="0" selectUnlockedCells="1"/>
@@ -1387,57 +1383,53 @@
       </c>
     </row>
     <row r="3" spans="3:16384">
-      <c r="G3" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="H3">
-        <v>15</v>
+      <c r="G3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H3" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="3:16384">
       <c r="G4" t="s">
-        <v>5</v>
-      </c>
-      <c r="H4" t="s">
-        <v>23</v>
+        <v>6</v>
+      </c>
+      <c r="H4">
+        <f>MIN(A3:A619)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="3:16384">
       <c r="G5" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H5">
-        <f>MIN(A3:A619)</f>
+        <f>MAX(A3:A619)</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="3:16384">
       <c r="G6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H6">
-        <f>MAX(A3:A619)</f>
+        <f>COUNT(A3:A619)</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="3:16384">
       <c r="G7" t="s">
-        <v>8</v>
-      </c>
-      <c r="H7">
-        <f>COUNT(A3:A619)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="3:16384">
-      <c r="G8" t="s">
         <v>9</v>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>D . F . Edwards, in Handbook of Optical Constants of Solids, edited by E. D. Palik (Academic, Orlando, 1985), pp. 547-569.</t>
         </is>
       </c>
+    </row>
+    <row r="8" spans="3:16384">
+      <c r="G8" s="0"/>
+      <c r="H8" s="0"/>
     </row>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" selectLockedCells="1" sort="0" autoFilter="0" pivotTables="0" selectUnlockedCells="1"/>
@@ -19956,13 +19948,11 @@
       <c r="B3">
         <v>0.01007833</v>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Optical permittivity:</t>
-        </is>
-      </c>
-      <c r="H3">
-        <v>2.04</v>
+      <c r="G3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H3" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -19973,48 +19963,40 @@
         <v>1200.556</v>
       </c>
       <c r="G4" t="s">
-        <v>5</v>
-      </c>
-      <c r="H4" t="s">
-        <v>20</v>
+        <v>6</v>
+      </c>
+      <c r="H4">
+        <v>833</v>
       </c>
     </row>
     <row r="5" spans="1:8">
       <c r="G5" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H5">
-        <v>833</v>
+        <v>66667</v>
       </c>
     </row>
     <row r="6" spans="1:8">
       <c r="G6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H6">
-        <v>66667</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:8">
       <c r="G7" t="s">
-        <v>8</v>
-      </c>
-      <c r="H7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8">
-      <c r="G8" t="s">
         <v>9</v>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>I. H. Malitson, Applied Optics 2, 1103-1107 (1963)</t>
         </is>
       </c>
     </row>
-    <row r="9" spans="1:8">
-      <c r="H9" t="inlineStr">
+    <row r="8" spans="1:8">
+      <c r="H8" t="inlineStr">
         <is>
           <t>Sellmeier coefficients for CaF2, valid 0.15-12 microns</t>
         </is>
@@ -20580,52 +20562,48 @@
       </c>
     </row>
     <row r="3" spans="3:16384">
-      <c r="G3" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="H3">
-        <v>2</v>
+      <c r="G3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H3" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="3:16384">
       <c r="G4" t="s">
-        <v>5</v>
-      </c>
-      <c r="H4" t="s">
-        <v>23</v>
+        <v>6</v>
+      </c>
+      <c r="H4">
+        <f>MIN(A3:A619)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="3:16384">
       <c r="G5" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H5">
-        <f>MIN(A3:A619)</f>
+        <f>MAX(A3:A619)</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="3:16384">
       <c r="G6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H6">
-        <f>MAX(A3:A619)</f>
+        <f>COUNT(A3:A619)</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="3:16384">
       <c r="G7" t="s">
-        <v>8</v>
-      </c>
-      <c r="H7">
-        <f>COUNT(A3:A619)</f>
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="3:16384">
-      <c r="G8" t="s">
-        <v>9</v>
-      </c>
+      <c r="G8" s="0"/>
+      <c r="H8" s="0"/>
     </row>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" selectLockedCells="1" sort="0" autoFilter="0" pivotTables="0" selectUnlockedCells="1"/>
@@ -20686,52 +20664,48 @@
       </c>
     </row>
     <row r="3" spans="3:16384">
-      <c r="G3" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="H3">
-        <v>1</v>
+      <c r="G3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H3" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="3:16384">
       <c r="G4" t="s">
-        <v>5</v>
-      </c>
-      <c r="H4" t="s">
-        <v>23</v>
+        <v>6</v>
+      </c>
+      <c r="H4">
+        <f>MIN(A3:A619)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="3:16384">
       <c r="G5" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H5">
-        <f>MIN(A3:A619)</f>
+        <f>MAX(A3:A619)</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="3:16384">
       <c r="G6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H6">
-        <f>MAX(A3:A619)</f>
+        <f>COUNT(A3:A619)</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="3:16384">
       <c r="G7" t="s">
-        <v>8</v>
-      </c>
-      <c r="H7">
-        <f>COUNT(A3:A619)</f>
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="3:16384">
-      <c r="G8" t="s">
-        <v>9</v>
-      </c>
+      <c r="G8" s="0"/>
+      <c r="H8" s="0"/>
     </row>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" selectLockedCells="1" sort="0" autoFilter="0" pivotTables="0" selectUnlockedCells="1"/>
@@ -20792,52 +20766,48 @@
       </c>
     </row>
     <row r="3" spans="3:16384">
-      <c r="G3" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="H3">
-        <v>1</v>
+      <c r="G3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H3" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="3:16384">
       <c r="G4" t="s">
-        <v>5</v>
-      </c>
-      <c r="H4" t="s">
-        <v>23</v>
+        <v>6</v>
+      </c>
+      <c r="H4">
+        <f>MIN(A3:A619)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="3:16384">
       <c r="G5" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H5">
-        <f>MIN(A3:A619)</f>
+        <f>MAX(A3:A619)</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="3:16384">
       <c r="G6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H6">
-        <f>MAX(A3:A619)</f>
+        <f>COUNT(A3:A619)</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="3:16384">
       <c r="G7" t="s">
-        <v>8</v>
-      </c>
-      <c r="H7">
-        <f>COUNT(A3:A619)</f>
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="3:16384">
-      <c r="G8" t="s">
-        <v>9</v>
-      </c>
+      <c r="G8" s="0"/>
+      <c r="H8" s="0"/>
     </row>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" selectLockedCells="1" sort="0" autoFilter="0" pivotTables="0" selectUnlockedCells="1"/>
@@ -20898,52 +20868,48 @@
       </c>
     </row>
     <row r="3" spans="3:16384">
-      <c r="G3" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="H3">
-        <v>2.2799999999999998</v>
+      <c r="G3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H3" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="3:16384">
       <c r="G4" t="s">
-        <v>5</v>
-      </c>
-      <c r="H4" t="s">
-        <v>23</v>
+        <v>6</v>
+      </c>
+      <c r="H4">
+        <f>MIN(A3:A619)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="3:16384">
       <c r="G5" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H5">
-        <f>MIN(A3:A619)</f>
+        <f>MAX(A3:A619)</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="3:16384">
       <c r="G6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H6">
-        <f>MAX(A3:A619)</f>
+        <f>COUNT(A3:A619)</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="3:16384">
       <c r="G7" t="s">
-        <v>8</v>
-      </c>
-      <c r="H7">
-        <f>COUNT(A3:A619)</f>
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="3:16384">
-      <c r="G8" t="s">
-        <v>9</v>
-      </c>
+      <c r="G8" s="0"/>
+      <c r="H8" s="0"/>
     </row>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" selectLockedCells="1" sort="0" autoFilter="0" pivotTables="0" selectUnlockedCells="1"/>
@@ -21004,52 +20970,49 @@
       </c>
     </row>
     <row r="3" spans="3:16384">
-      <c r="G3" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="H3">
-        <v>2.2999999999999998</v>
+      <c r="G3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H3" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="3:16384">
       <c r="G4" t="s">
-        <v>5</v>
-      </c>
-      <c r="H4" t="s">
-        <v>23</v>
+        <v>6</v>
+      </c>
+      <c r="H4">
+        <f>MIN(A3:A619)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="3:16384">
       <c r="G5" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H5">
-        <f>MIN(A3:A619)</f>
+        <f>MAX(A3:A619)</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="3:16384">
       <c r="G6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H6">
-        <f>MAX(A3:A619)</f>
+        <f>COUNT(A3:A619)</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="3:16384">
       <c r="G7" t="s">
-        <v>8</v>
-      </c>
-      <c r="H7">
-        <f>COUNT(A3:A619)</f>
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="3:16384">
-      <c r="G8" t="s">
-        <v>9</v>
-      </c>
+      <c r="G8" s="0"/>
+      <c r="H8" s="0"/>
+      <c r="I8" s="0"/>
     </row>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" selectLockedCells="1" sort="0" autoFilter="0" pivotTables="0" selectUnlockedCells="1"/>
@@ -21110,52 +21073,48 @@
       </c>
     </row>
     <row r="3" spans="3:16384">
-      <c r="G3" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="H3">
-        <v>4.9000000000000004</v>
+      <c r="G3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H3" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="3:16384">
       <c r="G4" t="s">
-        <v>5</v>
-      </c>
-      <c r="H4" t="s">
-        <v>23</v>
+        <v>6</v>
+      </c>
+      <c r="H4">
+        <f>MIN(A3:A619)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="3:16384">
       <c r="G5" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H5">
-        <f>MIN(A3:A619)</f>
+        <f>MAX(A3:A619)</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="3:16384">
       <c r="G6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H6">
-        <f>MAX(A3:A619)</f>
+        <f>COUNT(A3:A619)</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="3:16384">
       <c r="G7" t="s">
-        <v>8</v>
-      </c>
-      <c r="H7">
-        <f>COUNT(A3:A619)</f>
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="3:16384">
-      <c r="G8" t="s">
-        <v>9</v>
-      </c>
+      <c r="G8" s="0"/>
+      <c r="H8" s="0"/>
     </row>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" selectLockedCells="1" sort="0" autoFilter="0" pivotTables="0" selectUnlockedCells="1"/>
@@ -21216,52 +21175,48 @@
       </c>
     </row>
     <row r="3" spans="3:16384">
-      <c r="G3" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="H3">
-        <v>2.1499999999999999</v>
+      <c r="G3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H3" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="3:16384">
       <c r="G4" t="s">
-        <v>5</v>
-      </c>
-      <c r="H4" t="s">
-        <v>23</v>
+        <v>6</v>
+      </c>
+      <c r="H4">
+        <f>MIN(A3:A619)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="3:16384">
       <c r="G5" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H5">
-        <f>MIN(A3:A619)</f>
+        <f>MAX(A3:A619)</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="3:16384">
       <c r="G6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H6">
-        <f>MAX(A3:A619)</f>
+        <f>COUNT(A3:A619)</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="3:16384">
       <c r="G7" t="s">
-        <v>8</v>
-      </c>
-      <c r="H7">
-        <f>COUNT(A3:A619)</f>
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="3:16384">
-      <c r="G8" t="s">
-        <v>9</v>
-      </c>
+      <c r="G8" s="0"/>
+      <c r="H8" s="0"/>
     </row>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" selectLockedCells="1" sort="0" autoFilter="0" pivotTables="0" selectUnlockedCells="1"/>

</xml_diff>